<commit_message>
Auto commit (2026-09-23 16:24) — 2 changes
Claude Code 세션 종료 시 자동 커밋.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/dcabaf86-74c5-4e55-8ffe-3e508ca493e2
</commit_message>
<xml_diff>
--- a/projects/16_moses/내 남편은 거지 모세_CD1 셀링 포인트_v4.xlsx
+++ b/projects/16_moses/내 남편은 거지 모세_CD1 셀링 포인트_v4.xlsx
@@ -23059,12 +23059,18 @@
       </c>
       <c r="B17" s="243" t="inlineStr">
         <is>
-          <t>굴욕 장면 바로 뒤에 그 값을 치르는 장면이 붙어 있다. 발을 씻긴 뒤에는 이 떼가, 라반이 맞은 뒤에는 우박이 오고, 얼굴에 낙인이 닿기 직전에는 모래폭풍이 막아선다. 18화에서는 델릴라와 파라오의 얼굴이 다말이 걸었던 불길 앞으로 끌려간다. 바다는 두 번 갈라진다. 7화 혼례 날 지참금 망신 바로 뒤에 한 번, 46~47화 백성이 바다를 건널 때 또 한 번. 델릴라 몸에 개구리와 이가 들러붙는 장면은 우습게 쓰여 있다. 델릴라가 무너지는 장면은 34·35·49화에 세 번 나온다.</t>
+          <t>· 굴욕 바로 뒤에 되갚는 장면이 붙어 있다: 발 씻기 뒤 이 떼 / 라반 구타 뒤 우박 / 낙인 직전 모래폭풍 / 18화 델릴라·파라오 얼굴을 불길 앞으로.
+· 바다 가르기 두 번: 7화(지참금 망신 직후), 46~47화(백성이 건너는 장면).
+· 델릴라가 무너지는 장면 세 번: 34·35·49화.
+· 개구리·이 장면은 웃기게 쓰여 있다.</t>
         </is>
       </c>
       <c r="C17" s="243" t="inlineStr">
         <is>
-          <t>Every humiliation is followed right away by its payback: lice after the foot-washing, hail after Laban is beaten, and a sandstorm right before the branding iron lands. In EP18 Delilah and Pharaoh have their faces dragged to the same fire Tamar walked through. The sea parts twice: once in EP7, right after the dowry humiliation on the wedding day, and again in EP46-47 when the people cross. The frogs and lice crawling over Delilah are written for laughs. Delilah's fall happens three separate times, in EP34, EP35 and EP49.</t>
+          <t>· Every humiliation is followed right away by payback: lice after the foot-washing / hail after Laban is beaten / a sandstorm right before the brand lands / EP18 Delilah and Pharaoh's faces dragged to the fire.
+· The sea parts twice: EP7 (right after the dowry humiliation) and EP46-47 (the people cross).
+· Delilah falls three times: EP34, EP35, EP49.
+· The frogs and lice scenes are written for laughs.</t>
         </is>
       </c>
       <c r="F17" s="247" t="n">
@@ -23559,8 +23565,12 @@
       </c>
       <c r="B34" s="243" t="inlineStr">
         <is>
-          <t>동생 에리스와 함께 회귀한 아이린이 조용히 살려고 아무도 없는 쪽으로 화관을 던지는데, 에리스가 등을 떠밀어 화관이 남루한 떠돌이 음유시인의 손에 떨어지는 장면. 지난 생에 에리스가 엮였던 바로 그 남자다. 혼례 날 에리스의 지참금으로 금화 아흔아홉 상자가 공개되고 천 주머니 하나뿐인 아이린이 비웃음을 사는데, 오지 않던 신랑이 "내 신부를 맞으러 왔다"는 목소리와 함께 나타나는 장면. 아이린을 괴롭히던 가족들이 그 음유시인이 빛의 신 아폴론이라는 걸 먼저 알고 바닥에 엎드리는 장면. 아폴론의 어머니 레토 여신이 둘의 혼인을 반대하며 아이린을 신전 하녀로 시험하고, 아폴론은 정체도 힘도 쓰지 못한 채 경비병으로 변장해 곁을 지키는 장면. 모든 시련을 견딘 아이린이 그제야 남편이 아폴론이라는 걸 알게 되는 장면(44화). 끝까지 언니를 해치려던 에리스가 용암 감옥에 사슬로 묶인 채 언니와 마주하는 장면(46화).
-각색은 이 흐름을 그대로 따르면서 화관을 비둘기로, 아폴론을 예언자 모세로, 신의 힘을 열 가지 재앙과 바다 가르기로 바꿨다. 모세와 출애굽, 열 가지 재앙은 기독교 문화에 익숙한 서구권 시청자라면 설명 없이도 아는 이야기라, 그리스 신화보다 쉽게 다가간다.</t>
+          <t>① 동생이 등을 떠밀어, 언니의 화관이 거지 음유시인 손에 떨어진다.
+② 지참금 망신을 당하는 혼례 날, 하늘에서 "내 신부를 맞으러 왔다".
+③ 그 거지가 빛의 신 아폴론이라는 걸 가족들이 먼저 알고 바닥에 엎드린다.
+④ 아내만 모른다. 시어머니 여신의 시험을 다 견딘 뒤에야 안다(44화).
+⑤ 언니를 해치려던 동생은 용암 감옥에 사슬로 묶인다(46화).
+각색: 화관은 비둘기로, 아폴론은 모세로, 신의 힘은 열 가지 재앙과 바다 가르기로 바꿨다. 모세·출애굽·열 가지 재앙은 서구권 시청자가 이미 아는 이야기다.</t>
         </is>
       </c>
       <c r="C34" s="243" t="n"/>

</xml_diff>

<commit_message>
Auto commit (2026-09-23 16:35) — 2 changes
Claude Code 세션 종료 시 자동 커밋.

Co-Authored-By: Claude <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/0b9c28ed-17d6-46a9-b519-059f3d6e0a51
</commit_message>
<xml_diff>
--- a/projects/16_moses/내 남편은 거지 모세_CD1 셀링 포인트_v4.xlsx
+++ b/projects/16_moses/내 남편은 거지 모세_CD1 셀링 포인트_v4.xlsx
@@ -22699,7 +22699,7 @@
       </c>
       <c r="H4" s="243" t="inlineStr">
         <is>
-          <t>대왕비 책봉식에서 두루마리를 받아 든 다말의 등에 델릴라가 단검을 박아 넣는다. 델릴라는 3년 전 같은 날 새 날리기 의식에서 자신은 거지와 엮였는데 다말만 파라오를 얻었다며 울부짖고, 불기둥이 델릴라까지 집어삼켜 두 사람이 나란히 숨을 거둔다. 다말이 3년 전 새 날리기 의식 날 아침으로 돌아와 눈을 뜨고, 이번 생의 파라오는 자기가 갖겠다는 델릴라의 귓속말을 듣고 델릴라도 같은 날로 돌아왔음을 알아챈다. 델릴라가 먼저 황금 새장의 매를 잡아 파라오에게 날려 보내고, 매가 파라오의 어깨에 앉자 가족들이 환호한다.</t>
+          <t>대왕비 책봉식에서 두루마리를 받아 든 다말의 등에 델릴라가 단검을 박아 넣는다. 델릴라는 3년 전 같은 날 새 날리기 의식에서 자신은 거지와 엮였는데 다말만 파라오를 얻었다며 울부짖고, 불기둥이 델릴라를 집어삼키고, 두 사람이 나란히 숨을 거둔다. 다말이 3년 전 새 날리기 의식 날 아침으로 돌아와 눈을 뜨고, 이번 생의 파라오는 자기가 갖겠다는 델릴라의 귓속말을 듣고 델릴라도 같은 날로 돌아왔음을 알아챈다. 델릴라가 먼저 황금 새장의 매를 잡아 파라오에게 날려 보내고, 매가 파라오의 어깨에 앉자 가족들이 환호한다.</t>
         </is>
       </c>
     </row>
@@ -23238,7 +23238,7 @@
       </c>
       <c r="B23" s="243" t="inlineStr">
         <is>
-          <t>라반 가문의 큰딸. 전생에 파라오의 아내로 살다 대왕비로 책봉되던 날 이복동생의 단검에 죽었고, 3년 전 배필을 정하는 새 의식 아침으로 돌아왔다. 이번에는 아무도 없는 쪽으로 비둘기를 날리는데, 비둘기가 노예 구역의 거지 모세에게 가 앉자 가족 앞에서 그를 남편으로 받아들인다. 뺨을 맞고, 맨발로 불 위를 걷고, 동생의 발을 씻기고, 목에 칼이 들어와도 남편을 부르지 않는다. 그리고 다말을 괴롭힌 사람들에게 재앙이 하나씩 떨어진다. 광고로 쓸 만한 장면은 대부분 다말에게서 나온다.</t>
+          <t>라반 가문의 큰딸. 전생에 파라오의 아내로 살다 대왕비로 책봉되던 날 이복동생의 단검에 죽었고, 3년 전 배필을 정하는 새 의식 아침으로 돌아왔다. 이번에는 아무도 없는 쪽으로 비둘기를 날리는데, 비둘기가 노예 구역의 거지 모세에게 가 앉자 가족 앞에서 그를 남편으로 받아들인다. 뺨을 맞고, 맨발로 불 위를 걷고, 동생의 발을 씻기고, 목에 칼이 들어와도 남편을 부르지 않는다. 그리고 다말을 괴롭힌 사람들에게 모세의 재앙이 하나씩 떨어진다. 광고로 쓸 만한 장면은 대부분 다말에게서 나온다.</t>
         </is>
       </c>
       <c r="C23" s="243" t="inlineStr">
@@ -23310,7 +23310,7 @@
       </c>
       <c r="B25" s="243" t="inlineStr">
         <is>
-          <t>다말의 이복동생. 전생에 거지와 엮여 비참하게 살다가 언니를 죽였고, 같은 날로 함께 회귀해 이번에는 파라오를 먼저 채간다. 언니를 자기보다 더 비참하게 만드는 것이 목표다. 펜던트를 미끼로 언니를 맨발로 불 위를 걷게 하고 달군 낙인을 얼굴에 내리찍으려 하고(EP15~16), 감옥에서 무릎 꿇려 발을 씻긴다(EP28). 개구리가 방을 뒤덮고(EP24), 발을 씻긴 새벽에는 이가 몸에 들러붙고(EP28), 광장에서는 우박에 맞는다(EP30). EP34에서 파라오가 다말에게 대왕비 관을 내밀자 근위병에게 끌려 나가고, EP49에서 바다에 휩쓸린 뒤 진흙 속에서 다말의 발치까지 기어오지만 다말이 그 손목의 대왕비 팔찌를 빼내 웅덩이에 던진다. 죽지도 못한 채 살아서 죗값을 치른다.</t>
+          <t>다말의 이복동생. 전생에 거지와 엮여 비참하게 살다가 언니를 죽였고, 같은 날로 함께 회귀해 이번에는 파라오를 먼저 채간다. 언니를 자기보다 더 비참하게 만드는 것이 목표다. 펜던트를 미끼로 언니를 맨발로 불 위를 걷게 하고 달군 낙인을 얼굴에 내리찍으려 하고(EP15~16), 감옥에서 언니를 무릎 꿇려 자기 발을 씻기게 한다(EP28). 개구리가 방을 뒤덮고(EP24), 발을 씻긴 새벽에는 이가 몸에 들러붙고(EP28), 광장에서는 우박에 맞는다(EP30). EP34에서 파라오가 다말에게 대왕비 관을 내밀자 근위병에게 끌려 나가고, EP49에서 바다에 휩쓸린 뒤 진흙 속에서 다말의 발치까지 기어오지만 다말이 그 손목의 대왕비 팔찌를 빼내 웅덩이에 던진다. 죽지도 못한 채 살아서 죗값을 치른다.</t>
         </is>
       </c>
       <c r="C25" s="243" t="inlineStr">

</xml_diff>